<commit_message>
CRUD cursos ok, correción de visualizacion de usuarios.php
</commit_message>
<xml_diff>
--- a/archivos_soporte/Documentos/E-DO-ST-F 038 LISTA DE BRIGADISTAS-Institucin Educativa Tcnica Valle de Tenza.xlsx
+++ b/archivos_soporte/Documentos/E-DO-ST-F 038 LISTA DE BRIGADISTAS-Institucin Educativa Tcnica Valle de Tenza.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2026\Proyectos Transversales\fase II\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laravel\redvital_colvatenza\archivos_soporte\Documentos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7955231D-BBCB-457A-965E-E510F855A3AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBE6A5A4-9389-4ECF-93BE-5D952C3A2BB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CONTRAINCENDIOS" sheetId="1" r:id="rId1"/>
@@ -18,9 +18,9 @@
     <sheet name="EVACUACION Y RESCATE" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">CONTRAINCENDIOS!$B$8:$KG$86</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'EVACUACION Y RESCATE'!$B$8:$KG$85</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'PRIMEROS AUXILIOS'!$B$8:$KG$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">CONTRAINCENDIOS!$B$8:$H$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'EVACUACION Y RESCATE'!$B$8:$H$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'PRIMEROS AUXILIOS'!$B$8:$H$23</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -755,7 +755,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="20">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -1007,27 +1007,12 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1119,6 +1104,67 @@
     <xf numFmtId="15" fontId="11" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1170,75 +1216,23 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="6" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="9" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1662,83 +1656,83 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B1:I53"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="15" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.5546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="23.109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="3.5703125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="23.140625" style="1" customWidth="1"/>
     <col min="3" max="3" width="23" style="1" customWidth="1"/>
-    <col min="4" max="4" width="20.33203125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="18.88671875" style="13" customWidth="1"/>
-    <col min="6" max="6" width="49.5546875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="33.6640625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="36.6640625" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="11.44140625" style="1"/>
+    <col min="4" max="4" width="20.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="18.85546875" style="13" customWidth="1"/>
+    <col min="6" max="6" width="49.5703125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="33.7109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="36.7109375" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:9" ht="15.6" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="2:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="38"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="46" t="s">
+    <row r="1" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="59"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="67" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
       <c r="H2" s="14" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="2:9" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="40"/>
-      <c r="C3" s="41"/>
-      <c r="D3" s="47"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="47"/>
-      <c r="G3" s="47"/>
+    <row r="3" spans="2:9" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="61"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="68"/>
+      <c r="E3" s="68"/>
+      <c r="F3" s="68"/>
+      <c r="G3" s="68"/>
       <c r="H3" s="15" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="2:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="44" t="s">
+    <row r="4" spans="2:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="45"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="45"/>
-      <c r="G4" s="45"/>
+      <c r="C4" s="66"/>
+      <c r="D4" s="66"/>
+      <c r="E4" s="66"/>
+      <c r="F4" s="66"/>
+      <c r="G4" s="66"/>
       <c r="H4" s="28" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="2:9" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="42" t="s">
+    <row r="5" spans="2:9" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="43"/>
-      <c r="D5" s="43"/>
-      <c r="E5" s="43"/>
-      <c r="F5" s="43"/>
-      <c r="G5" s="43"/>
-      <c r="H5" s="43"/>
+      <c r="C5" s="64"/>
+      <c r="D5" s="64"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64"/>
+      <c r="G5" s="64"/>
+      <c r="H5" s="64"/>
       <c r="I5" s="16"/>
     </row>
-    <row r="6" spans="2:9" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="36" t="s">
+    <row r="6" spans="2:9" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="37"/>
-      <c r="D6" s="34" t="s">
+      <c r="C6" s="58"/>
+      <c r="D6" s="55" t="s">
         <v>172</v>
       </c>
-      <c r="E6" s="34"/>
-      <c r="F6" s="35"/>
+      <c r="E6" s="55"/>
+      <c r="F6" s="56"/>
       <c r="G6" s="29" t="s">
         <v>11</v>
       </c>
@@ -1747,17 +1741,17 @@
       </c>
       <c r="I6" s="16"/>
     </row>
-    <row r="7" spans="2:9" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="B7" s="31"/>
-      <c r="C7" s="32"/>
-      <c r="D7" s="32"/>
-      <c r="E7" s="32"/>
-      <c r="F7" s="32"/>
-      <c r="G7" s="32"/>
-      <c r="H7" s="33"/>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B7" s="52"/>
+      <c r="C7" s="53"/>
+      <c r="D7" s="53"/>
+      <c r="E7" s="53"/>
+      <c r="F7" s="53"/>
+      <c r="G7" s="53"/>
+      <c r="H7" s="54"/>
       <c r="I7" s="16"/>
     </row>
-    <row r="8" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B8" s="17" t="s">
         <v>0</v>
       </c>
@@ -1780,375 +1774,375 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:9" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="67" t="s">
+    <row r="9" spans="2:9" s="37" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="47" t="s">
         <v>53</v>
       </c>
-      <c r="C9" s="48" t="s">
+      <c r="C9" s="31" t="s">
         <v>54</v>
       </c>
-      <c r="D9" s="68">
+      <c r="D9" s="48">
         <v>4130645</v>
       </c>
-      <c r="E9" s="69" t="s">
+      <c r="E9" s="49" t="s">
         <v>52</v>
       </c>
-      <c r="F9" s="48" t="s">
+      <c r="F9" s="31" t="s">
         <v>36</v>
       </c>
-      <c r="G9" s="48" t="s">
+      <c r="G9" s="31" t="s">
         <v>55</v>
       </c>
-      <c r="H9" s="70" t="s">
+      <c r="H9" s="50" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="2:9" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="67" t="s">
+    <row r="10" spans="2:9" s="37" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="47" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="48" t="s">
+      <c r="C10" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="D10" s="68">
+      <c r="D10" s="48">
         <v>1049795764</v>
       </c>
-      <c r="E10" s="69" t="s">
+      <c r="E10" s="49" t="s">
         <v>34</v>
       </c>
-      <c r="F10" s="48" t="s">
+      <c r="F10" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="G10" s="48" t="s">
+      <c r="G10" s="31" t="s">
         <v>139</v>
       </c>
-      <c r="H10" s="70" t="s">
+      <c r="H10" s="50" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="2:9" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="67" t="s">
+    <row r="11" spans="2:9" s="37" customFormat="1" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="47" t="s">
         <v>188</v>
       </c>
-      <c r="C11" s="48" t="s">
+      <c r="C11" s="31" t="s">
         <v>189</v>
       </c>
-      <c r="D11" s="68">
+      <c r="D11" s="48">
         <v>1002737008</v>
       </c>
-      <c r="E11" s="69" t="s">
+      <c r="E11" s="49" t="s">
         <v>190</v>
       </c>
-      <c r="F11" s="71" t="s">
+      <c r="F11" s="51" t="s">
         <v>191</v>
       </c>
-      <c r="G11" s="48" t="s">
+      <c r="G11" s="31" t="s">
         <v>139</v>
       </c>
-      <c r="H11" s="70" t="s">
+      <c r="H11" s="50" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="12" spans="2:9" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="67" t="s">
+    <row r="12" spans="2:9" s="37" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="47" t="s">
         <v>37</v>
       </c>
-      <c r="C12" s="48" t="s">
+      <c r="C12" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="D12" s="68">
+      <c r="D12" s="48">
         <v>1010162722</v>
       </c>
-      <c r="E12" s="69" t="s">
+      <c r="E12" s="49" t="s">
         <v>39</v>
       </c>
-      <c r="F12" s="48" t="s">
+      <c r="F12" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="G12" s="48" t="s">
+      <c r="G12" s="31" t="s">
         <v>139</v>
       </c>
-      <c r="H12" s="70" t="s">
+      <c r="H12" s="50" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="2:9" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="67" t="s">
+    <row r="13" spans="2:9" s="37" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="47" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="48" t="s">
+      <c r="C13" s="31" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="68">
+      <c r="D13" s="48">
         <v>74282470</v>
       </c>
-      <c r="E13" s="69" t="s">
+      <c r="E13" s="49" t="s">
         <v>50</v>
       </c>
-      <c r="F13" s="48" t="s">
+      <c r="F13" s="31" t="s">
         <v>51</v>
       </c>
-      <c r="G13" s="48" t="s">
+      <c r="G13" s="31" t="s">
         <v>139</v>
       </c>
-      <c r="H13" s="70" t="s">
+      <c r="H13" s="50" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="2:9" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="67" t="s">
+    <row r="14" spans="2:9" s="37" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="48" t="s">
+      <c r="C14" s="31" t="s">
         <v>62</v>
       </c>
-      <c r="D14" s="68">
+      <c r="D14" s="48">
         <v>6768269</v>
       </c>
-      <c r="E14" s="69">
+      <c r="E14" s="49">
         <v>3193925032</v>
       </c>
-      <c r="F14" s="48" t="s">
+      <c r="F14" s="31" t="s">
         <v>63</v>
       </c>
-      <c r="G14" s="48" t="s">
+      <c r="G14" s="31" t="s">
         <v>139</v>
       </c>
-      <c r="H14" s="70" t="s">
+      <c r="H14" s="50" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="2:9" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="67" t="s">
+    <row r="15" spans="2:9" s="37" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="47" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="48" t="s">
+      <c r="C15" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="D15" s="68">
+      <c r="D15" s="48">
         <v>1054658587</v>
       </c>
-      <c r="E15" s="69" t="s">
+      <c r="E15" s="49" t="s">
         <v>43</v>
       </c>
-      <c r="F15" s="48" t="s">
+      <c r="F15" s="31" t="s">
         <v>44</v>
       </c>
-      <c r="G15" s="48" t="s">
+      <c r="G15" s="31" t="s">
         <v>139</v>
       </c>
-      <c r="H15" s="70" t="s">
+      <c r="H15" s="50" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="2:9" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="67" t="s">
+    <row r="16" spans="2:9" s="37" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="47" t="s">
         <v>88</v>
       </c>
-      <c r="C16" s="48" t="s">
+      <c r="C16" s="31" t="s">
         <v>89</v>
       </c>
-      <c r="D16" s="68">
+      <c r="D16" s="48">
         <v>40020480</v>
       </c>
-      <c r="E16" s="69" t="s">
+      <c r="E16" s="49" t="s">
         <v>45</v>
       </c>
-      <c r="F16" s="48" t="s">
+      <c r="F16" s="31" t="s">
         <v>46</v>
       </c>
-      <c r="G16" s="48" t="s">
+      <c r="G16" s="31" t="s">
         <v>47</v>
       </c>
-      <c r="H16" s="70" t="s">
+      <c r="H16" s="50" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="2:8" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="67" t="s">
+    <row r="17" spans="2:8" s="37" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="47" t="s">
         <v>22</v>
       </c>
-      <c r="C17" s="48" t="s">
+      <c r="C17" s="31" t="s">
         <v>64</v>
       </c>
-      <c r="D17" s="68">
+      <c r="D17" s="48">
         <v>33367121</v>
       </c>
-      <c r="E17" s="69">
+      <c r="E17" s="49">
         <v>3028379174</v>
       </c>
-      <c r="F17" s="48" t="s">
+      <c r="F17" s="31" t="s">
         <v>65</v>
       </c>
-      <c r="G17" s="48" t="s">
+      <c r="G17" s="31" t="s">
         <v>139</v>
       </c>
-      <c r="H17" s="70" t="s">
+      <c r="H17" s="50" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="2:8" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="67" t="s">
+    <row r="18" spans="2:8" s="37" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="47" t="s">
         <v>15</v>
       </c>
-      <c r="C18" s="48" t="s">
+      <c r="C18" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="D18" s="68">
+      <c r="D18" s="48">
         <v>40013291</v>
       </c>
-      <c r="E18" s="69" t="s">
+      <c r="E18" s="49" t="s">
         <v>30</v>
       </c>
-      <c r="F18" s="48" t="s">
+      <c r="F18" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="G18" s="48" t="s">
+      <c r="G18" s="31" t="s">
         <v>139</v>
       </c>
-      <c r="H18" s="70" t="s">
+      <c r="H18" s="50" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="2:8" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="67" t="s">
+    <row r="19" spans="2:8" s="37" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="47" t="s">
         <v>90</v>
       </c>
-      <c r="C19" s="48" t="s">
+      <c r="C19" s="31" t="s">
         <v>91</v>
       </c>
-      <c r="D19" s="68">
+      <c r="D19" s="48">
         <v>24138150</v>
       </c>
-      <c r="E19" s="69" t="s">
+      <c r="E19" s="49" t="s">
         <v>48</v>
       </c>
-      <c r="F19" s="48" t="s">
+      <c r="F19" s="31" t="s">
         <v>134</v>
       </c>
-      <c r="G19" s="48" t="s">
+      <c r="G19" s="31" t="s">
         <v>49</v>
       </c>
-      <c r="H19" s="70" t="s">
+      <c r="H19" s="50" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="2:8" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="67" t="s">
+    <row r="20" spans="2:8" s="37" customFormat="1" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="47" t="s">
         <v>184</v>
       </c>
-      <c r="C20" s="48" t="s">
+      <c r="C20" s="31" t="s">
         <v>185</v>
       </c>
-      <c r="D20" s="68">
+      <c r="D20" s="48">
         <v>40038432</v>
       </c>
-      <c r="E20" s="69" t="s">
+      <c r="E20" s="49" t="s">
         <v>186</v>
       </c>
-      <c r="F20" s="48" t="s">
+      <c r="F20" s="31" t="s">
         <v>187</v>
       </c>
-      <c r="G20" s="48" t="s">
+      <c r="G20" s="31" t="s">
         <v>139</v>
       </c>
-      <c r="H20" s="70" t="s">
+      <c r="H20" s="50" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="21" spans="2:8" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="67" t="s">
+    <row r="21" spans="2:8" s="37" customFormat="1" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="47" t="s">
         <v>152</v>
       </c>
-      <c r="C21" s="48" t="s">
+      <c r="C21" s="31" t="s">
         <v>153</v>
       </c>
-      <c r="D21" s="68">
+      <c r="D21" s="48">
         <v>28169085</v>
       </c>
-      <c r="E21" s="69" t="s">
+      <c r="E21" s="49" t="s">
         <v>154</v>
       </c>
-      <c r="F21" s="48" t="s">
+      <c r="F21" s="31" t="s">
         <v>155</v>
       </c>
-      <c r="G21" s="48" t="s">
+      <c r="G21" s="31" t="s">
         <v>139</v>
       </c>
-      <c r="H21" s="70" t="s">
+      <c r="H21" s="50" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="22" spans="2:8" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="67" t="s">
+    <row r="22" spans="2:8" s="37" customFormat="1" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="47" t="s">
         <v>163</v>
       </c>
-      <c r="C22" s="48" t="s">
+      <c r="C22" s="31" t="s">
         <v>164</v>
       </c>
-      <c r="D22" s="68">
+      <c r="D22" s="48">
         <v>1056957376</v>
       </c>
-      <c r="E22" s="69">
+      <c r="E22" s="49">
         <v>3135803056</v>
       </c>
-      <c r="F22" s="48" t="s">
+      <c r="F22" s="31" t="s">
         <v>141</v>
       </c>
-      <c r="G22" s="48" t="s">
+      <c r="G22" s="31" t="s">
         <v>139</v>
       </c>
-      <c r="H22" s="70" t="s">
+      <c r="H22" s="50" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="23" spans="2:8" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="67" t="s">
+    <row r="23" spans="2:8" s="37" customFormat="1" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="47" t="s">
         <v>142</v>
       </c>
-      <c r="C23" s="48" t="s">
+      <c r="C23" s="31" t="s">
         <v>143</v>
       </c>
-      <c r="D23" s="68">
+      <c r="D23" s="48">
         <v>1048849296</v>
       </c>
-      <c r="E23" s="69">
+      <c r="E23" s="49">
         <v>3142791082</v>
       </c>
-      <c r="F23" s="48" t="s">
+      <c r="F23" s="31" t="s">
         <v>144</v>
       </c>
-      <c r="G23" s="48" t="s">
+      <c r="G23" s="31" t="s">
         <v>139</v>
       </c>
-      <c r="H23" s="70" t="s">
+      <c r="H23" s="50" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="24" spans="2:8" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="67" t="s">
+    <row r="24" spans="2:8" s="37" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="47" t="s">
         <v>192</v>
       </c>
-      <c r="C24" s="48" t="s">
+      <c r="C24" s="31" t="s">
         <v>193</v>
       </c>
-      <c r="D24" s="68">
+      <c r="D24" s="48">
         <v>46387482</v>
       </c>
-      <c r="E24" s="69">
+      <c r="E24" s="49">
         <v>3195270974</v>
       </c>
-      <c r="F24" s="48" t="s">
+      <c r="F24" s="31" t="s">
         <v>194</v>
       </c>
-      <c r="G24" s="48" t="s">
+      <c r="G24" s="31" t="s">
         <v>139</v>
       </c>
-      <c r="H24" s="70" t="s">
+      <c r="H24" s="50" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="25" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="19"/>
       <c r="C25" s="3"/>
       <c r="D25" s="5"/>
@@ -2157,7 +2151,7 @@
       <c r="G25" s="3"/>
       <c r="H25" s="23"/>
     </row>
-    <row r="26" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="19"/>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
@@ -2166,7 +2160,7 @@
       <c r="G26" s="3"/>
       <c r="H26" s="24"/>
     </row>
-    <row r="27" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="19"/>
       <c r="C27" s="3"/>
       <c r="D27" s="4"/>
@@ -2175,7 +2169,7 @@
       <c r="G27" s="3"/>
       <c r="H27" s="23"/>
     </row>
-    <row r="28" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="19"/>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
@@ -2184,7 +2178,7 @@
       <c r="G28" s="3"/>
       <c r="H28" s="25"/>
     </row>
-    <row r="29" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="19"/>
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
@@ -2193,7 +2187,7 @@
       <c r="G29" s="3"/>
       <c r="H29" s="23"/>
     </row>
-    <row r="30" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="19"/>
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
@@ -2202,7 +2196,7 @@
       <c r="G30" s="3"/>
       <c r="H30" s="23"/>
     </row>
-    <row r="31" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="19"/>
       <c r="C31" s="3"/>
       <c r="D31" s="4"/>
@@ -2211,7 +2205,7 @@
       <c r="G31" s="3"/>
       <c r="H31" s="22"/>
     </row>
-    <row r="32" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="19"/>
       <c r="C32" s="3"/>
       <c r="D32" s="4"/>
@@ -2220,7 +2214,7 @@
       <c r="G32" s="3"/>
       <c r="H32" s="21"/>
     </row>
-    <row r="33" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="19"/>
       <c r="C33" s="3"/>
       <c r="D33" s="5"/>
@@ -2229,7 +2223,7 @@
       <c r="G33" s="3"/>
       <c r="H33" s="26"/>
     </row>
-    <row r="34" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="19"/>
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
@@ -2238,7 +2232,7 @@
       <c r="G34" s="3"/>
       <c r="H34" s="21"/>
     </row>
-    <row r="35" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="19"/>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
@@ -2247,7 +2241,7 @@
       <c r="G35" s="3"/>
       <c r="H35" s="22"/>
     </row>
-    <row r="36" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="19"/>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
@@ -2256,7 +2250,7 @@
       <c r="G36" s="3"/>
       <c r="H36" s="21"/>
     </row>
-    <row r="37" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="19"/>
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
@@ -2265,7 +2259,7 @@
       <c r="G37" s="3"/>
       <c r="H37" s="24"/>
     </row>
-    <row r="38" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="19"/>
       <c r="C38" s="3"/>
       <c r="D38" s="3"/>
@@ -2274,7 +2268,7 @@
       <c r="G38" s="3"/>
       <c r="H38" s="21"/>
     </row>
-    <row r="39" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="19"/>
       <c r="C39" s="3"/>
       <c r="D39" s="4"/>
@@ -2283,7 +2277,7 @@
       <c r="G39" s="3"/>
       <c r="H39" s="23"/>
     </row>
-    <row r="40" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="19"/>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
@@ -2292,7 +2286,7 @@
       <c r="G40" s="3"/>
       <c r="H40" s="21"/>
     </row>
-    <row r="41" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="19"/>
       <c r="C41" s="3"/>
       <c r="D41" s="5"/>
@@ -2301,7 +2295,7 @@
       <c r="G41" s="3"/>
       <c r="H41" s="23"/>
     </row>
-    <row r="42" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B42" s="19"/>
       <c r="C42" s="3"/>
       <c r="D42" s="4"/>
@@ -2310,7 +2304,7 @@
       <c r="G42" s="3"/>
       <c r="H42" s="22"/>
     </row>
-    <row r="43" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="19"/>
       <c r="C43" s="3"/>
       <c r="D43" s="5"/>
@@ -2319,7 +2313,7 @@
       <c r="G43" s="3"/>
       <c r="H43" s="23"/>
     </row>
-    <row r="44" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B44" s="19"/>
       <c r="C44" s="3"/>
       <c r="D44" s="4"/>
@@ -2328,7 +2322,7 @@
       <c r="G44" s="3"/>
       <c r="H44" s="23"/>
     </row>
-    <row r="45" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="19"/>
       <c r="C45" s="3"/>
       <c r="D45" s="3"/>
@@ -2337,7 +2331,7 @@
       <c r="G45" s="3"/>
       <c r="H45" s="23"/>
     </row>
-    <row r="46" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="27"/>
       <c r="C46" s="6"/>
       <c r="D46" s="6"/>
@@ -2346,7 +2340,7 @@
       <c r="G46" s="3"/>
       <c r="H46" s="20"/>
     </row>
-    <row r="47" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="19"/>
       <c r="C47" s="3"/>
       <c r="D47" s="3"/>
@@ -2355,7 +2349,7 @@
       <c r="G47" s="3"/>
       <c r="H47" s="23"/>
     </row>
-    <row r="48" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B48" s="19"/>
       <c r="C48" s="3"/>
       <c r="D48" s="4"/>
@@ -2364,7 +2358,7 @@
       <c r="G48" s="3"/>
       <c r="H48" s="21"/>
     </row>
-    <row r="49" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="19"/>
       <c r="C49" s="3"/>
       <c r="D49" s="5"/>
@@ -2373,7 +2367,7 @@
       <c r="G49" s="3"/>
       <c r="H49" s="23"/>
     </row>
-    <row r="50" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B50" s="19"/>
       <c r="C50" s="3"/>
       <c r="D50" s="3"/>
@@ -2382,7 +2376,7 @@
       <c r="G50" s="3"/>
       <c r="H50" s="21"/>
     </row>
-    <row r="51" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B51" s="19"/>
       <c r="C51" s="3"/>
       <c r="D51" s="5"/>
@@ -2391,7 +2385,7 @@
       <c r="G51" s="11"/>
       <c r="H51" s="22"/>
     </row>
-    <row r="52" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B52" s="19"/>
       <c r="C52" s="3"/>
       <c r="D52" s="4"/>
@@ -2400,8 +2394,15 @@
       <c r="G52" s="3"/>
       <c r="H52" s="20"/>
     </row>
-    <row r="53" spans="2:8" ht="27" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="53" spans="2:8" ht="27" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
+  <autoFilter ref="B8:H24" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="6">
+      <filters>
+        <filter val="Campestre"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B9:I23">
     <sortCondition ref="B9:B23"/>
   </sortState>
@@ -2440,83 +2441,83 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B1:I51"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="15" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.5546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="23.109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="3.5703125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="23.140625" style="1" customWidth="1"/>
     <col min="3" max="3" width="23" style="1" customWidth="1"/>
-    <col min="4" max="4" width="20.33203125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="18.88671875" style="13" customWidth="1"/>
-    <col min="6" max="6" width="49.5546875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="33.6640625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="36.6640625" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="11.44140625" style="1"/>
+    <col min="4" max="4" width="20.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="18.85546875" style="13" customWidth="1"/>
+    <col min="6" max="6" width="49.5703125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="33.7109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="36.7109375" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:9" ht="15.6" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="2:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="38"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="46" t="s">
+    <row r="1" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="59"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="67" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
       <c r="H2" s="14" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="2:9" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="40"/>
-      <c r="C3" s="41"/>
-      <c r="D3" s="47"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="47"/>
-      <c r="G3" s="47"/>
+    <row r="3" spans="2:9" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="61"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="68"/>
+      <c r="E3" s="68"/>
+      <c r="F3" s="68"/>
+      <c r="G3" s="68"/>
       <c r="H3" s="15" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="2:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="44" t="s">
+    <row r="4" spans="2:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="45"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="45"/>
-      <c r="G4" s="45"/>
+      <c r="C4" s="66"/>
+      <c r="D4" s="66"/>
+      <c r="E4" s="66"/>
+      <c r="F4" s="66"/>
+      <c r="G4" s="66"/>
       <c r="H4" s="28" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="2:9" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="42" t="s">
+    <row r="5" spans="2:9" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="63" t="s">
         <v>96</v>
       </c>
-      <c r="C5" s="43"/>
-      <c r="D5" s="43"/>
-      <c r="E5" s="43"/>
-      <c r="F5" s="43"/>
-      <c r="G5" s="43"/>
-      <c r="H5" s="43"/>
+      <c r="C5" s="64"/>
+      <c r="D5" s="64"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64"/>
+      <c r="G5" s="64"/>
+      <c r="H5" s="64"/>
       <c r="I5" s="16"/>
     </row>
-    <row r="6" spans="2:9" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="36" t="s">
+    <row r="6" spans="2:9" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="37"/>
-      <c r="D6" s="34" t="s">
+      <c r="C6" s="58"/>
+      <c r="D6" s="55" t="s">
         <v>172</v>
       </c>
-      <c r="E6" s="34"/>
-      <c r="F6" s="35"/>
+      <c r="E6" s="55"/>
+      <c r="F6" s="56"/>
       <c r="G6" s="29" t="s">
         <v>11</v>
       </c>
@@ -2525,17 +2526,17 @@
       </c>
       <c r="I6" s="16"/>
     </row>
-    <row r="7" spans="2:9" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="B7" s="31"/>
-      <c r="C7" s="32"/>
-      <c r="D7" s="32"/>
-      <c r="E7" s="32"/>
-      <c r="F7" s="32"/>
-      <c r="G7" s="32"/>
-      <c r="H7" s="33"/>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B7" s="52"/>
+      <c r="C7" s="53"/>
+      <c r="D7" s="53"/>
+      <c r="E7" s="53"/>
+      <c r="F7" s="53"/>
+      <c r="G7" s="53"/>
+      <c r="H7" s="54"/>
       <c r="I7" s="16"/>
     </row>
-    <row r="8" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B8" s="17" t="s">
         <v>0</v>
       </c>
@@ -2558,596 +2559,603 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:9" s="54" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="56" t="s">
+    <row r="9" spans="2:9" s="37" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="56" t="s">
+      <c r="C9" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="57">
+      <c r="D9" s="40">
         <v>52528519</v>
       </c>
-      <c r="E9" s="58">
+      <c r="E9" s="41">
         <v>3102685590</v>
       </c>
-      <c r="F9" s="59" t="s">
+      <c r="F9" s="42" t="s">
         <v>56</v>
       </c>
-      <c r="G9" s="56" t="s">
+      <c r="G9" s="39" t="s">
         <v>57</v>
       </c>
-      <c r="H9" s="56" t="s">
+      <c r="H9" s="39" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="2:9" s="54" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="56" t="s">
+    <row r="10" spans="2:9" s="37" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="56" t="s">
+      <c r="C10" s="39" t="s">
         <v>60</v>
       </c>
-      <c r="D10" s="57">
+      <c r="D10" s="40">
         <v>23323550</v>
       </c>
-      <c r="E10" s="58">
+      <c r="E10" s="41">
         <v>3134943767</v>
       </c>
-      <c r="F10" s="59" t="s">
+      <c r="F10" s="42" t="s">
         <v>59</v>
       </c>
-      <c r="G10" s="56" t="s">
+      <c r="G10" s="39" t="s">
         <v>139</v>
       </c>
-      <c r="H10" s="56" t="s">
+      <c r="H10" s="39" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="2:9" s="54" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="52" t="s">
+    <row r="11" spans="2:9" s="37" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="35" t="s">
         <v>180</v>
       </c>
-      <c r="C11" s="52" t="s">
+      <c r="C11" s="35" t="s">
         <v>181</v>
       </c>
-      <c r="D11" s="60">
+      <c r="D11" s="43">
         <v>40047973</v>
       </c>
-      <c r="E11" s="58" t="s">
+      <c r="E11" s="41" t="s">
         <v>182</v>
       </c>
-      <c r="F11" s="51" t="s">
+      <c r="F11" s="34" t="s">
         <v>183</v>
       </c>
-      <c r="G11" s="52" t="s">
+      <c r="G11" s="35" t="s">
         <v>139</v>
       </c>
-      <c r="H11" s="61" t="s">
+      <c r="H11" s="44" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="2:9" s="54" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="56" t="s">
+    <row r="12" spans="2:9" s="37" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="39" t="s">
         <v>82</v>
       </c>
-      <c r="C12" s="56" t="s">
+      <c r="C12" s="39" t="s">
         <v>83</v>
       </c>
-      <c r="D12" s="57">
+      <c r="D12" s="40">
         <v>24138789</v>
       </c>
-      <c r="E12" s="58" t="s">
+      <c r="E12" s="41" t="s">
         <v>84</v>
       </c>
-      <c r="F12" s="59" t="s">
+      <c r="F12" s="42" t="s">
         <v>85</v>
       </c>
-      <c r="G12" s="56" t="s">
+      <c r="G12" s="39" t="s">
         <v>86</v>
       </c>
-      <c r="H12" s="56" t="s">
+      <c r="H12" s="39" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="2:9" s="54" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="56" t="s">
+    <row r="13" spans="2:9" s="37" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="39" t="s">
         <v>72</v>
       </c>
-      <c r="C13" s="56" t="s">
+      <c r="C13" s="39" t="s">
         <v>73</v>
       </c>
-      <c r="D13" s="57">
+      <c r="D13" s="40">
         <v>1052386533</v>
       </c>
-      <c r="E13" s="58">
+      <c r="E13" s="41">
         <v>3125763008</v>
       </c>
-      <c r="F13" s="59" t="s">
+      <c r="F13" s="42" t="s">
         <v>74</v>
       </c>
-      <c r="G13" s="56" t="s">
+      <c r="G13" s="39" t="s">
         <v>139</v>
       </c>
-      <c r="H13" s="56" t="s">
+      <c r="H13" s="39" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="2:9" s="54" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="56" t="s">
+    <row r="14" spans="2:9" s="37" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="39" t="s">
         <v>160</v>
       </c>
-      <c r="C14" s="56" t="s">
+      <c r="C14" s="39" t="s">
         <v>161</v>
       </c>
-      <c r="D14" s="57">
+      <c r="D14" s="40">
         <v>33703159</v>
       </c>
-      <c r="E14" s="58">
+      <c r="E14" s="41">
         <v>3045591758</v>
       </c>
-      <c r="F14" s="59" t="s">
+      <c r="F14" s="42" t="s">
         <v>162</v>
       </c>
-      <c r="G14" s="56" t="s">
+      <c r="G14" s="39" t="s">
         <v>139</v>
       </c>
-      <c r="H14" s="56" t="s">
+      <c r="H14" s="39" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="2:9" s="54" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="56" t="s">
+    <row r="15" spans="2:9" s="37" customFormat="1" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="39" t="s">
         <v>156</v>
       </c>
-      <c r="C15" s="56" t="s">
+      <c r="C15" s="39" t="s">
         <v>157</v>
       </c>
-      <c r="D15" s="57">
+      <c r="D15" s="40">
         <v>23622716</v>
       </c>
-      <c r="E15" s="58" t="s">
+      <c r="E15" s="41" t="s">
         <v>158</v>
       </c>
-      <c r="F15" s="59" t="s">
+      <c r="F15" s="42" t="s">
         <v>159</v>
       </c>
-      <c r="G15" s="56" t="s">
+      <c r="G15" s="39" t="s">
         <v>139</v>
       </c>
-      <c r="H15" s="62" t="s">
+      <c r="H15" s="45" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="16" spans="2:9" s="54" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="56" t="s">
+    <row r="16" spans="2:9" s="37" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="39" t="s">
         <v>69</v>
       </c>
-      <c r="C16" s="56" t="s">
+      <c r="C16" s="39" t="s">
         <v>70</v>
       </c>
-      <c r="D16" s="57">
+      <c r="D16" s="40">
         <v>80100466</v>
       </c>
-      <c r="E16" s="58">
+      <c r="E16" s="41">
         <v>3212426214</v>
       </c>
-      <c r="F16" s="59" t="s">
+      <c r="F16" s="42" t="s">
         <v>71</v>
       </c>
-      <c r="G16" s="56" t="s">
+      <c r="G16" s="39" t="s">
         <v>139</v>
       </c>
-      <c r="H16" s="56" t="s">
+      <c r="H16" s="39" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="2:8" s="54" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="52" t="s">
+    <row r="17" spans="2:8" s="37" customFormat="1" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="35" t="s">
         <v>169</v>
       </c>
-      <c r="C17" s="52" t="s">
+      <c r="C17" s="35" t="s">
         <v>170</v>
       </c>
-      <c r="D17" s="57">
+      <c r="D17" s="40">
         <v>51942414</v>
       </c>
-      <c r="E17" s="63">
+      <c r="E17" s="46">
         <v>3213761852</v>
       </c>
-      <c r="F17" s="59" t="s">
+      <c r="F17" s="42" t="s">
         <v>171</v>
       </c>
-      <c r="G17" s="56" t="s">
+      <c r="G17" s="39" t="s">
         <v>139</v>
       </c>
-      <c r="H17" s="62" t="s">
+      <c r="H17" s="45" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="18" spans="2:8" s="54" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="56" t="s">
+    <row r="18" spans="2:8" s="37" customFormat="1" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="39" t="s">
         <v>92</v>
       </c>
-      <c r="C18" s="56" t="s">
+      <c r="C18" s="39" t="s">
         <v>93</v>
       </c>
-      <c r="D18" s="57">
+      <c r="D18" s="40">
         <v>40048003</v>
       </c>
-      <c r="E18" s="58" t="s">
+      <c r="E18" s="41" t="s">
         <v>94</v>
       </c>
-      <c r="F18" s="59" t="s">
+      <c r="F18" s="42" t="s">
         <v>95</v>
       </c>
-      <c r="G18" s="56" t="s">
+      <c r="G18" s="39" t="s">
         <v>139</v>
       </c>
-      <c r="H18" s="62" t="s">
+      <c r="H18" s="45" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="19" spans="2:8" s="54" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="56" t="s">
+    <row r="19" spans="2:8" s="37" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="39" t="s">
         <v>75</v>
       </c>
-      <c r="C19" s="56" t="s">
+      <c r="C19" s="39" t="s">
         <v>76</v>
       </c>
-      <c r="D19" s="57">
+      <c r="D19" s="40">
         <v>1049609038</v>
       </c>
-      <c r="E19" s="58" t="s">
+      <c r="E19" s="41" t="s">
         <v>77</v>
       </c>
-      <c r="F19" s="59" t="s">
+      <c r="F19" s="42" t="s">
         <v>78</v>
       </c>
-      <c r="G19" s="56" t="s">
+      <c r="G19" s="39" t="s">
         <v>139</v>
       </c>
-      <c r="H19" s="56" t="s">
+      <c r="H19" s="39" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="2:8" s="54" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="56" t="s">
+    <row r="20" spans="2:8" s="37" customFormat="1" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="39" t="s">
         <v>97</v>
       </c>
-      <c r="C20" s="56" t="s">
+      <c r="C20" s="39" t="s">
         <v>79</v>
       </c>
-      <c r="D20" s="57">
+      <c r="D20" s="40">
         <v>1057185092</v>
       </c>
-      <c r="E20" s="58">
+      <c r="E20" s="41">
         <v>3133092962</v>
       </c>
-      <c r="F20" s="59" t="s">
+      <c r="F20" s="42" t="s">
         <v>80</v>
       </c>
-      <c r="G20" s="56" t="s">
+      <c r="G20" s="39" t="s">
         <v>139</v>
       </c>
-      <c r="H20" s="56" t="s">
+      <c r="H20" s="39" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="21" spans="2:8" s="54" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="56" t="s">
+    <row r="21" spans="2:8" s="37" customFormat="1" ht="27" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="39" t="s">
         <v>135</v>
       </c>
-      <c r="C21" s="56" t="s">
+      <c r="C21" s="39" t="s">
         <v>136</v>
       </c>
-      <c r="D21" s="57">
+      <c r="D21" s="40">
         <v>40022735</v>
       </c>
-      <c r="E21" s="58" t="s">
+      <c r="E21" s="41" t="s">
         <v>137</v>
       </c>
-      <c r="F21" s="59" t="s">
+      <c r="F21" s="42" t="s">
         <v>138</v>
       </c>
-      <c r="G21" s="56" t="s">
+      <c r="G21" s="39" t="s">
         <v>139</v>
       </c>
-      <c r="H21" s="62" t="s">
+      <c r="H21" s="45" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="22" spans="2:8" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="64" t="s">
+    <row r="22" spans="2:8" s="37" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="39" t="s">
         <v>66</v>
       </c>
-      <c r="C22" s="64" t="s">
+      <c r="C22" s="39" t="s">
         <v>67</v>
       </c>
-      <c r="D22" s="57">
+      <c r="D22" s="40">
         <v>74379934</v>
       </c>
-      <c r="E22" s="58">
+      <c r="E22" s="41">
         <v>3107511851</v>
       </c>
-      <c r="F22" s="59" t="s">
+      <c r="F22" s="42" t="s">
         <v>68</v>
       </c>
-      <c r="G22" s="56" t="s">
+      <c r="G22" s="39" t="s">
         <v>139</v>
       </c>
-      <c r="H22" s="56" t="s">
+      <c r="H22" s="39" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="23" spans="2:8" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="64" t="s">
+    <row r="23" spans="2:8" s="37" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="C23" s="56" t="s">
+      <c r="C23" s="39" t="s">
         <v>61</v>
       </c>
-      <c r="D23" s="65">
+      <c r="D23" s="40">
         <v>40027873</v>
       </c>
-      <c r="E23" s="58">
+      <c r="E23" s="41">
         <v>3213721875</v>
       </c>
-      <c r="F23" s="59" t="s">
+      <c r="F23" s="42" t="s">
         <v>58</v>
       </c>
-      <c r="G23" s="56" t="s">
+      <c r="G23" s="39" t="s">
         <v>139</v>
       </c>
-      <c r="H23" s="66" t="s">
+      <c r="H23" s="39" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="24" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="19"/>
+    <row r="24" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="3"/>
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
       <c r="E24" s="10"/>
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
-      <c r="H24" s="24"/>
-    </row>
-    <row r="25" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="19"/>
+      <c r="H24" s="69"/>
+    </row>
+    <row r="25" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="3"/>
       <c r="C25" s="3"/>
       <c r="D25" s="4"/>
       <c r="E25" s="8"/>
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
-      <c r="H25" s="23"/>
-    </row>
-    <row r="26" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="19"/>
+      <c r="H25" s="70"/>
+    </row>
+    <row r="26" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="3"/>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
       <c r="E26" s="8"/>
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
-      <c r="H26" s="25"/>
-    </row>
-    <row r="27" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="19"/>
+      <c r="H26" s="71"/>
+    </row>
+    <row r="27" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="3"/>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
       <c r="E27" s="8"/>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
-      <c r="H27" s="23"/>
-    </row>
-    <row r="28" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="19"/>
+      <c r="H27" s="70"/>
+    </row>
+    <row r="28" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="3"/>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
       <c r="E28" s="8"/>
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
-      <c r="H28" s="23"/>
-    </row>
-    <row r="29" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="19"/>
+      <c r="H28" s="70"/>
+    </row>
+    <row r="29" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="3"/>
       <c r="C29" s="3"/>
       <c r="D29" s="4"/>
       <c r="E29" s="12"/>
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
-      <c r="H29" s="22"/>
-    </row>
-    <row r="30" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="19"/>
+      <c r="H29" s="72"/>
+    </row>
+    <row r="30" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="3"/>
       <c r="C30" s="3"/>
       <c r="D30" s="4"/>
       <c r="E30" s="12"/>
       <c r="F30" s="3"/>
       <c r="G30" s="3"/>
-      <c r="H30" s="21"/>
-    </row>
-    <row r="31" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="19"/>
+      <c r="H30" s="73"/>
+    </row>
+    <row r="31" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="3"/>
       <c r="C31" s="3"/>
       <c r="D31" s="5"/>
       <c r="E31" s="8"/>
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
-      <c r="H31" s="26"/>
-    </row>
-    <row r="32" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="19"/>
+      <c r="H31" s="74"/>
+    </row>
+    <row r="32" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="3"/>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
       <c r="E32" s="9"/>
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
-      <c r="H32" s="21"/>
-    </row>
-    <row r="33" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="19"/>
+      <c r="H32" s="73"/>
+    </row>
+    <row r="33" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="3"/>
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
       <c r="E33" s="8"/>
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
-      <c r="H33" s="22"/>
-    </row>
-    <row r="34" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="19"/>
+      <c r="H33" s="72"/>
+    </row>
+    <row r="34" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="3"/>
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
       <c r="E34" s="9"/>
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
-      <c r="H34" s="21"/>
-    </row>
-    <row r="35" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="19"/>
+      <c r="H34" s="73"/>
+    </row>
+    <row r="35" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="3"/>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
       <c r="E35" s="9"/>
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
-      <c r="H35" s="24"/>
-    </row>
-    <row r="36" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="19"/>
+      <c r="H35" s="69"/>
+    </row>
+    <row r="36" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B36" s="3"/>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
       <c r="E36" s="9"/>
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
-      <c r="H36" s="21"/>
-    </row>
-    <row r="37" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="19"/>
+      <c r="H36" s="73"/>
+    </row>
+    <row r="37" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B37" s="3"/>
       <c r="C37" s="3"/>
       <c r="D37" s="4"/>
       <c r="E37" s="8"/>
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
-      <c r="H37" s="23"/>
-    </row>
-    <row r="38" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="19"/>
+      <c r="H37" s="70"/>
+    </row>
+    <row r="38" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="3"/>
       <c r="C38" s="3"/>
       <c r="D38" s="3"/>
       <c r="E38" s="9"/>
       <c r="F38" s="3"/>
       <c r="G38" s="3"/>
-      <c r="H38" s="21"/>
-    </row>
-    <row r="39" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="19"/>
+      <c r="H38" s="73"/>
+    </row>
+    <row r="39" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B39" s="3"/>
       <c r="C39" s="3"/>
       <c r="D39" s="5"/>
       <c r="E39" s="8"/>
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
-      <c r="H39" s="23"/>
-    </row>
-    <row r="40" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B40" s="19"/>
+      <c r="H39" s="70"/>
+    </row>
+    <row r="40" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B40" s="3"/>
       <c r="C40" s="3"/>
       <c r="D40" s="4"/>
       <c r="E40" s="8"/>
       <c r="F40" s="3"/>
       <c r="G40" s="3"/>
-      <c r="H40" s="22"/>
-    </row>
-    <row r="41" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B41" s="19"/>
+      <c r="H40" s="72"/>
+    </row>
+    <row r="41" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B41" s="3"/>
       <c r="C41" s="3"/>
       <c r="D41" s="5"/>
       <c r="E41" s="8"/>
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
-      <c r="H41" s="23"/>
-    </row>
-    <row r="42" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B42" s="19"/>
+      <c r="H41" s="70"/>
+    </row>
+    <row r="42" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B42" s="3"/>
       <c r="C42" s="3"/>
       <c r="D42" s="4"/>
       <c r="E42" s="8"/>
       <c r="F42" s="3"/>
       <c r="G42" s="3"/>
-      <c r="H42" s="23"/>
-    </row>
-    <row r="43" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B43" s="19"/>
+      <c r="H42" s="70"/>
+    </row>
+    <row r="43" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B43" s="3"/>
       <c r="C43" s="3"/>
       <c r="D43" s="3"/>
       <c r="E43" s="8"/>
       <c r="F43" s="3"/>
       <c r="G43" s="3"/>
-      <c r="H43" s="23"/>
-    </row>
-    <row r="44" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B44" s="27"/>
+      <c r="H43" s="70"/>
+    </row>
+    <row r="44" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B44" s="6"/>
       <c r="C44" s="6"/>
       <c r="D44" s="6"/>
       <c r="E44" s="10"/>
       <c r="F44" s="6"/>
       <c r="G44" s="3"/>
-      <c r="H44" s="20"/>
-    </row>
-    <row r="45" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B45" s="19"/>
+      <c r="H44" s="6"/>
+    </row>
+    <row r="45" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B45" s="3"/>
       <c r="C45" s="3"/>
       <c r="D45" s="3"/>
       <c r="E45" s="8"/>
       <c r="F45" s="3"/>
       <c r="G45" s="3"/>
-      <c r="H45" s="23"/>
-    </row>
-    <row r="46" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B46" s="19"/>
+      <c r="H45" s="70"/>
+    </row>
+    <row r="46" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B46" s="3"/>
       <c r="C46" s="3"/>
       <c r="D46" s="4"/>
       <c r="E46" s="12"/>
       <c r="F46" s="3"/>
       <c r="G46" s="3"/>
-      <c r="H46" s="21"/>
-    </row>
-    <row r="47" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B47" s="19"/>
+      <c r="H46" s="73"/>
+    </row>
+    <row r="47" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B47" s="3"/>
       <c r="C47" s="3"/>
       <c r="D47" s="5"/>
       <c r="E47" s="8"/>
       <c r="F47" s="3"/>
       <c r="G47" s="3"/>
-      <c r="H47" s="23"/>
-    </row>
-    <row r="48" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B48" s="19"/>
+      <c r="H47" s="70"/>
+    </row>
+    <row r="48" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B48" s="3"/>
       <c r="C48" s="3"/>
       <c r="D48" s="3"/>
       <c r="E48" s="9"/>
       <c r="F48" s="3"/>
       <c r="G48" s="3"/>
-      <c r="H48" s="21"/>
-    </row>
-    <row r="49" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B49" s="19"/>
+      <c r="H48" s="73"/>
+    </row>
+    <row r="49" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B49" s="3"/>
       <c r="C49" s="3"/>
       <c r="D49" s="5"/>
       <c r="E49" s="8"/>
       <c r="F49" s="3"/>
       <c r="G49" s="11"/>
-      <c r="H49" s="22"/>
-    </row>
-    <row r="50" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B50" s="19"/>
+      <c r="H49" s="72"/>
+    </row>
+    <row r="50" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B50" s="3"/>
       <c r="C50" s="3"/>
       <c r="D50" s="4"/>
       <c r="E50" s="8"/>
       <c r="F50" s="3"/>
       <c r="G50" s="3"/>
-      <c r="H50" s="20"/>
-    </row>
-    <row r="51" spans="2:8" ht="27" customHeight="1" x14ac:dyDescent="0.3"/>
+      <c r="H50" s="6"/>
+    </row>
+    <row r="51" spans="2:8" ht="27" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
+  <autoFilter ref="B8:H23" xr:uid="{00000000-0001-0000-0100-000000000000}">
+    <filterColumn colId="6">
+      <filters>
+        <filter val="Campestre"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B9:I23">
     <sortCondition ref="B9:B23"/>
   </sortState>
@@ -3183,83 +3191,83 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B1:I52"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="15" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.5546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="23.109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="3.5703125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="23.140625" style="1" customWidth="1"/>
     <col min="3" max="3" width="23" style="1" customWidth="1"/>
-    <col min="4" max="4" width="20.33203125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="18.88671875" style="13" customWidth="1"/>
-    <col min="6" max="6" width="49.5546875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="33.6640625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="36.6640625" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="11.44140625" style="1"/>
+    <col min="4" max="4" width="20.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="18.85546875" style="13" customWidth="1"/>
+    <col min="6" max="6" width="49.5703125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="33.7109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="36.7109375" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:9" ht="15.6" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="2:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="38"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="46" t="s">
+    <row r="1" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="59"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="67" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
       <c r="H2" s="14" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="2:9" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="40"/>
-      <c r="C3" s="41"/>
-      <c r="D3" s="47"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="47"/>
-      <c r="G3" s="47"/>
+    <row r="3" spans="2:9" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="61"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="68"/>
+      <c r="E3" s="68"/>
+      <c r="F3" s="68"/>
+      <c r="G3" s="68"/>
       <c r="H3" s="15" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="2:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="44" t="s">
+    <row r="4" spans="2:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="45"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="45"/>
-      <c r="G4" s="45"/>
+      <c r="C4" s="66"/>
+      <c r="D4" s="66"/>
+      <c r="E4" s="66"/>
+      <c r="F4" s="66"/>
+      <c r="G4" s="66"/>
       <c r="H4" s="28" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="2:9" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="42" t="s">
+    <row r="5" spans="2:9" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="43"/>
-      <c r="D5" s="43"/>
-      <c r="E5" s="43"/>
-      <c r="F5" s="43"/>
-      <c r="G5" s="43"/>
-      <c r="H5" s="43"/>
+      <c r="C5" s="64"/>
+      <c r="D5" s="64"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64"/>
+      <c r="G5" s="64"/>
+      <c r="H5" s="64"/>
       <c r="I5" s="16"/>
     </row>
-    <row r="6" spans="2:9" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="36" t="s">
+    <row r="6" spans="2:9" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="37"/>
-      <c r="D6" s="34" t="s">
+      <c r="C6" s="58"/>
+      <c r="D6" s="55" t="s">
         <v>172</v>
       </c>
-      <c r="E6" s="34"/>
-      <c r="F6" s="35"/>
+      <c r="E6" s="55"/>
+      <c r="F6" s="56"/>
       <c r="G6" s="29" t="s">
         <v>11</v>
       </c>
@@ -3268,17 +3276,17 @@
       </c>
       <c r="I6" s="16"/>
     </row>
-    <row r="7" spans="2:9" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="B7" s="31"/>
-      <c r="C7" s="32"/>
-      <c r="D7" s="32"/>
-      <c r="E7" s="32"/>
-      <c r="F7" s="32"/>
-      <c r="G7" s="32"/>
-      <c r="H7" s="33"/>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B7" s="52"/>
+      <c r="C7" s="53"/>
+      <c r="D7" s="53"/>
+      <c r="E7" s="53"/>
+      <c r="F7" s="53"/>
+      <c r="G7" s="53"/>
+      <c r="H7" s="54"/>
       <c r="I7" s="16"/>
     </row>
-    <row r="8" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B8" s="17" t="s">
         <v>0</v>
       </c>
@@ -3301,352 +3309,352 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:9" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="48" t="s">
+    <row r="9" spans="2:9" s="37" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B9" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="48" t="s">
+      <c r="C9" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="49">
+      <c r="D9" s="32">
         <v>4145435</v>
       </c>
-      <c r="E9" s="50" t="s">
+      <c r="E9" s="33" t="s">
         <v>126</v>
       </c>
-      <c r="F9" s="51" t="s">
+      <c r="F9" s="34" t="s">
         <v>168</v>
       </c>
-      <c r="G9" s="52" t="s">
+      <c r="G9" s="35" t="s">
         <v>127</v>
       </c>
-      <c r="H9" s="53" t="s">
+      <c r="H9" s="36" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="2:9" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="48" t="s">
+    <row r="10" spans="2:9" s="37" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B10" s="31" t="s">
         <v>87</v>
       </c>
-      <c r="C10" s="48" t="s">
+      <c r="C10" s="31" t="s">
         <v>98</v>
       </c>
-      <c r="D10" s="49">
+      <c r="D10" s="32">
         <v>74327211</v>
       </c>
-      <c r="E10" s="50" t="s">
+      <c r="E10" s="33" t="s">
         <v>99</v>
       </c>
-      <c r="F10" s="55" t="s">
+      <c r="F10" s="38" t="s">
         <v>100</v>
       </c>
-      <c r="G10" s="52" t="s">
+      <c r="G10" s="35" t="s">
         <v>101</v>
       </c>
-      <c r="H10" s="53" t="s">
+      <c r="H10" s="36" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="2:9" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="48" t="s">
+    <row r="11" spans="2:9" s="37" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B11" s="31" t="s">
         <v>109</v>
       </c>
-      <c r="C11" s="48" t="s">
+      <c r="C11" s="31" t="s">
         <v>110</v>
       </c>
-      <c r="D11" s="49">
+      <c r="D11" s="32">
         <v>9528120</v>
       </c>
-      <c r="E11" s="50" t="s">
+      <c r="E11" s="33" t="s">
         <v>111</v>
       </c>
-      <c r="F11" s="55" t="s">
+      <c r="F11" s="38" t="s">
         <v>102</v>
       </c>
-      <c r="G11" s="52" t="s">
+      <c r="G11" s="35" t="s">
         <v>139</v>
       </c>
-      <c r="H11" s="53" t="s">
+      <c r="H11" s="36" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="2:9" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="48" t="s">
+    <row r="12" spans="2:9" s="37" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B12" s="31" t="s">
         <v>176</v>
       </c>
-      <c r="C12" s="48" t="s">
+      <c r="C12" s="31" t="s">
         <v>177</v>
       </c>
-      <c r="D12" s="49">
+      <c r="D12" s="32">
         <v>4218163</v>
       </c>
-      <c r="E12" s="50" t="s">
+      <c r="E12" s="33" t="s">
         <v>178</v>
       </c>
-      <c r="F12" s="55" t="s">
+      <c r="F12" s="38" t="s">
         <v>179</v>
       </c>
-      <c r="G12" s="52" t="s">
+      <c r="G12" s="35" t="s">
         <v>139</v>
       </c>
-      <c r="H12" s="53" t="s">
+      <c r="H12" s="36" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="2:9" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="48" t="s">
+    <row r="13" spans="2:9" s="37" customFormat="1" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B13" s="31" t="s">
         <v>150</v>
       </c>
-      <c r="C13" s="48" t="s">
+      <c r="C13" s="31" t="s">
         <v>151</v>
       </c>
-      <c r="D13" s="49">
+      <c r="D13" s="32">
         <v>1018429250</v>
       </c>
-      <c r="E13" s="50" t="s">
+      <c r="E13" s="33" t="s">
         <v>140</v>
       </c>
-      <c r="F13" s="55" t="s">
+      <c r="F13" s="38" t="s">
         <v>149</v>
       </c>
-      <c r="G13" s="52" t="s">
+      <c r="G13" s="35" t="s">
         <v>139</v>
       </c>
-      <c r="H13" s="53" t="s">
+      <c r="H13" s="36" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="14" spans="2:9" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="48" t="s">
+    <row r="14" spans="2:9" s="37" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B14" s="31" t="s">
         <v>112</v>
       </c>
-      <c r="C14" s="48" t="s">
+      <c r="C14" s="31" t="s">
         <v>113</v>
       </c>
-      <c r="D14" s="49">
+      <c r="D14" s="32">
         <v>33365671</v>
       </c>
-      <c r="E14" s="50" t="s">
+      <c r="E14" s="33" t="s">
         <v>114</v>
       </c>
-      <c r="F14" s="55" t="s">
+      <c r="F14" s="38" t="s">
         <v>103</v>
       </c>
-      <c r="G14" s="52" t="s">
+      <c r="G14" s="35" t="s">
         <v>139</v>
       </c>
-      <c r="H14" s="53" t="s">
+      <c r="H14" s="36" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="2:9" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="48" t="s">
+    <row r="15" spans="2:9" s="37" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B15" s="31" t="s">
         <v>122</v>
       </c>
-      <c r="C15" s="48" t="s">
+      <c r="C15" s="31" t="s">
         <v>123</v>
       </c>
-      <c r="D15" s="49">
+      <c r="D15" s="32">
         <v>80222928</v>
       </c>
-      <c r="E15" s="50" t="s">
+      <c r="E15" s="33" t="s">
         <v>124</v>
       </c>
-      <c r="F15" s="55" t="s">
+      <c r="F15" s="38" t="s">
         <v>125</v>
       </c>
-      <c r="G15" s="52" t="s">
+      <c r="G15" s="35" t="s">
         <v>139</v>
       </c>
-      <c r="H15" s="53" t="s">
+      <c r="H15" s="36" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="2:9" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="48" t="s">
+    <row r="16" spans="2:9" s="37" customFormat="1" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="31" t="s">
         <v>165</v>
       </c>
-      <c r="C16" s="48" t="s">
+      <c r="C16" s="31" t="s">
         <v>166</v>
       </c>
-      <c r="D16" s="49">
+      <c r="D16" s="32">
         <v>1049610081</v>
       </c>
-      <c r="E16" s="50">
+      <c r="E16" s="33">
         <v>3203239112</v>
       </c>
-      <c r="F16" s="55" t="s">
+      <c r="F16" s="38" t="s">
         <v>167</v>
       </c>
-      <c r="G16" s="52" t="s">
+      <c r="G16" s="35" t="s">
         <v>139</v>
       </c>
-      <c r="H16" s="53" t="s">
+      <c r="H16" s="36" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="17" spans="2:8" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="48" t="s">
+    <row r="17" spans="2:8" s="37" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B17" s="31" t="s">
         <v>128</v>
       </c>
-      <c r="C17" s="48" t="s">
+      <c r="C17" s="31" t="s">
         <v>129</v>
       </c>
-      <c r="D17" s="49">
+      <c r="D17" s="32">
         <v>7332099</v>
       </c>
-      <c r="E17" s="50">
+      <c r="E17" s="33">
         <v>3223069258</v>
       </c>
-      <c r="F17" s="55" t="s">
+      <c r="F17" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="G17" s="52" t="s">
+      <c r="G17" s="35" t="s">
         <v>127</v>
       </c>
-      <c r="H17" s="53" t="s">
+      <c r="H17" s="36" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="2:8" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="48" t="s">
+    <row r="18" spans="2:8" s="37" customFormat="1" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B18" s="31" t="s">
         <v>145</v>
       </c>
-      <c r="C18" s="48" t="s">
+      <c r="C18" s="31" t="s">
         <v>146</v>
       </c>
-      <c r="D18" s="49">
+      <c r="D18" s="32">
         <v>1049798821</v>
       </c>
-      <c r="E18" s="50" t="s">
+      <c r="E18" s="33" t="s">
         <v>147</v>
       </c>
-      <c r="F18" s="55" t="s">
+      <c r="F18" s="38" t="s">
         <v>148</v>
       </c>
-      <c r="G18" s="52" t="s">
+      <c r="G18" s="35" t="s">
         <v>139</v>
       </c>
-      <c r="H18" s="53" t="s">
+      <c r="H18" s="36" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="19" spans="2:8" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="48" t="s">
+    <row r="19" spans="2:8" s="37" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B19" s="31" t="s">
         <v>116</v>
       </c>
-      <c r="C19" s="48" t="s">
+      <c r="C19" s="31" t="s">
         <v>115</v>
       </c>
-      <c r="D19" s="49">
+      <c r="D19" s="32">
         <v>23438430</v>
       </c>
-      <c r="E19" s="50" t="s">
+      <c r="E19" s="33" t="s">
         <v>117</v>
       </c>
-      <c r="F19" s="55" t="s">
+      <c r="F19" s="38" t="s">
         <v>118</v>
       </c>
-      <c r="G19" s="52" t="s">
+      <c r="G19" s="35" t="s">
         <v>139</v>
       </c>
-      <c r="H19" s="53" t="s">
+      <c r="H19" s="36" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="2:8" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="48" t="s">
+    <row r="20" spans="2:8" s="37" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B20" s="31" t="s">
         <v>131</v>
       </c>
-      <c r="C20" s="48" t="s">
+      <c r="C20" s="31" t="s">
         <v>132</v>
       </c>
-      <c r="D20" s="49">
+      <c r="D20" s="32">
         <v>1049622089</v>
       </c>
-      <c r="E20" s="50" t="s">
+      <c r="E20" s="33" t="s">
         <v>133</v>
       </c>
-      <c r="F20" s="55" t="s">
+      <c r="F20" s="38" t="s">
         <v>104</v>
       </c>
-      <c r="G20" s="52" t="s">
+      <c r="G20" s="35" t="s">
         <v>139</v>
       </c>
-      <c r="H20" s="53" t="s">
+      <c r="H20" s="36" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="2:8" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="48" t="s">
+    <row r="21" spans="2:8" s="37" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B21" s="31" t="s">
         <v>105</v>
       </c>
-      <c r="C21" s="48" t="s">
+      <c r="C21" s="31" t="s">
         <v>106</v>
       </c>
-      <c r="D21" s="49">
+      <c r="D21" s="32">
         <v>1033688051</v>
       </c>
-      <c r="E21" s="50" t="s">
+      <c r="E21" s="33" t="s">
         <v>107</v>
       </c>
-      <c r="F21" s="55" t="s">
+      <c r="F21" s="38" t="s">
         <v>108</v>
       </c>
-      <c r="G21" s="52" t="s">
+      <c r="G21" s="35" t="s">
         <v>139</v>
       </c>
-      <c r="H21" s="53" t="s">
+      <c r="H21" s="36" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="22" spans="2:8" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="48" t="s">
+    <row r="22" spans="2:8" s="37" customFormat="1" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B22" s="31" t="s">
         <v>173</v>
       </c>
-      <c r="C22" s="48" t="s">
+      <c r="C22" s="31" t="s">
         <v>174</v>
       </c>
-      <c r="D22" s="49">
+      <c r="D22" s="32">
         <v>4134295</v>
       </c>
-      <c r="E22" s="50">
+      <c r="E22" s="33">
         <v>3142736122</v>
       </c>
-      <c r="F22" s="55" t="s">
+      <c r="F22" s="38" t="s">
         <v>175</v>
       </c>
-      <c r="G22" s="52" t="s">
+      <c r="G22" s="35" t="s">
         <v>139</v>
       </c>
-      <c r="H22" s="53" t="s">
+      <c r="H22" s="36" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="23" spans="2:8" s="54" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="48" t="s">
+    <row r="23" spans="2:8" s="37" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B23" s="31" t="s">
         <v>24</v>
       </c>
-      <c r="C23" s="48" t="s">
+      <c r="C23" s="31" t="s">
         <v>119</v>
       </c>
-      <c r="D23" s="49">
+      <c r="D23" s="32">
         <v>52165782</v>
       </c>
-      <c r="E23" s="50" t="s">
+      <c r="E23" s="33" t="s">
         <v>120</v>
       </c>
-      <c r="F23" s="55" t="s">
+      <c r="F23" s="38" t="s">
         <v>121</v>
       </c>
-      <c r="G23" s="52" t="s">
+      <c r="G23" s="35" t="s">
         <v>139</v>
       </c>
-      <c r="H23" s="53" t="s">
+      <c r="H23" s="36" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="24" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="19"/>
       <c r="C24" s="3"/>
       <c r="D24" s="5"/>
@@ -3655,7 +3663,7 @@
       <c r="G24" s="3"/>
       <c r="H24" s="23"/>
     </row>
-    <row r="25" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="19"/>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
@@ -3664,7 +3672,7 @@
       <c r="G25" s="3"/>
       <c r="H25" s="24"/>
     </row>
-    <row r="26" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="19"/>
       <c r="C26" s="3"/>
       <c r="D26" s="4"/>
@@ -3673,7 +3681,7 @@
       <c r="G26" s="3"/>
       <c r="H26" s="23"/>
     </row>
-    <row r="27" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="19"/>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
@@ -3682,7 +3690,7 @@
       <c r="G27" s="3"/>
       <c r="H27" s="25"/>
     </row>
-    <row r="28" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="19"/>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
@@ -3691,7 +3699,7 @@
       <c r="G28" s="3"/>
       <c r="H28" s="23"/>
     </row>
-    <row r="29" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="19"/>
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
@@ -3700,7 +3708,7 @@
       <c r="G29" s="3"/>
       <c r="H29" s="23"/>
     </row>
-    <row r="30" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="19"/>
       <c r="C30" s="3"/>
       <c r="D30" s="4"/>
@@ -3709,7 +3717,7 @@
       <c r="G30" s="3"/>
       <c r="H30" s="22"/>
     </row>
-    <row r="31" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="19"/>
       <c r="C31" s="3"/>
       <c r="D31" s="4"/>
@@ -3718,7 +3726,7 @@
       <c r="G31" s="3"/>
       <c r="H31" s="21"/>
     </row>
-    <row r="32" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="19"/>
       <c r="C32" s="3"/>
       <c r="D32" s="5"/>
@@ -3727,7 +3735,7 @@
       <c r="G32" s="3"/>
       <c r="H32" s="26"/>
     </row>
-    <row r="33" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="19"/>
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
@@ -3736,7 +3744,7 @@
       <c r="G33" s="3"/>
       <c r="H33" s="21"/>
     </row>
-    <row r="34" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="19"/>
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
@@ -3745,7 +3753,7 @@
       <c r="G34" s="3"/>
       <c r="H34" s="22"/>
     </row>
-    <row r="35" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="19"/>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
@@ -3754,7 +3762,7 @@
       <c r="G35" s="3"/>
       <c r="H35" s="21"/>
     </row>
-    <row r="36" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="19"/>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
@@ -3763,7 +3771,7 @@
       <c r="G36" s="3"/>
       <c r="H36" s="24"/>
     </row>
-    <row r="37" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="19"/>
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
@@ -3772,7 +3780,7 @@
       <c r="G37" s="3"/>
       <c r="H37" s="21"/>
     </row>
-    <row r="38" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="19"/>
       <c r="C38" s="3"/>
       <c r="D38" s="4"/>
@@ -3781,7 +3789,7 @@
       <c r="G38" s="3"/>
       <c r="H38" s="23"/>
     </row>
-    <row r="39" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="19"/>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
@@ -3790,7 +3798,7 @@
       <c r="G39" s="3"/>
       <c r="H39" s="21"/>
     </row>
-    <row r="40" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="19"/>
       <c r="C40" s="3"/>
       <c r="D40" s="5"/>
@@ -3799,7 +3807,7 @@
       <c r="G40" s="3"/>
       <c r="H40" s="23"/>
     </row>
-    <row r="41" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="19"/>
       <c r="C41" s="3"/>
       <c r="D41" s="4"/>
@@ -3808,7 +3816,7 @@
       <c r="G41" s="3"/>
       <c r="H41" s="22"/>
     </row>
-    <row r="42" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B42" s="19"/>
       <c r="C42" s="3"/>
       <c r="D42" s="5"/>
@@ -3817,7 +3825,7 @@
       <c r="G42" s="3"/>
       <c r="H42" s="23"/>
     </row>
-    <row r="43" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="19"/>
       <c r="C43" s="3"/>
       <c r="D43" s="4"/>
@@ -3826,7 +3834,7 @@
       <c r="G43" s="3"/>
       <c r="H43" s="23"/>
     </row>
-    <row r="44" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B44" s="19"/>
       <c r="C44" s="3"/>
       <c r="D44" s="3"/>
@@ -3835,7 +3843,7 @@
       <c r="G44" s="3"/>
       <c r="H44" s="23"/>
     </row>
-    <row r="45" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="27"/>
       <c r="C45" s="6"/>
       <c r="D45" s="6"/>
@@ -3844,7 +3852,7 @@
       <c r="G45" s="3"/>
       <c r="H45" s="20"/>
     </row>
-    <row r="46" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="19"/>
       <c r="C46" s="3"/>
       <c r="D46" s="3"/>
@@ -3853,7 +3861,7 @@
       <c r="G46" s="3"/>
       <c r="H46" s="23"/>
     </row>
-    <row r="47" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="19"/>
       <c r="C47" s="3"/>
       <c r="D47" s="4"/>
@@ -3862,7 +3870,7 @@
       <c r="G47" s="3"/>
       <c r="H47" s="21"/>
     </row>
-    <row r="48" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B48" s="19"/>
       <c r="C48" s="3"/>
       <c r="D48" s="5"/>
@@ -3871,7 +3879,7 @@
       <c r="G48" s="3"/>
       <c r="H48" s="23"/>
     </row>
-    <row r="49" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="19"/>
       <c r="C49" s="3"/>
       <c r="D49" s="3"/>
@@ -3880,7 +3888,7 @@
       <c r="G49" s="3"/>
       <c r="H49" s="21"/>
     </row>
-    <row r="50" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B50" s="19"/>
       <c r="C50" s="3"/>
       <c r="D50" s="5"/>
@@ -3889,7 +3897,7 @@
       <c r="G50" s="11"/>
       <c r="H50" s="22"/>
     </row>
-    <row r="51" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B51" s="19"/>
       <c r="C51" s="3"/>
       <c r="D51" s="4"/>
@@ -3898,8 +3906,15 @@
       <c r="G51" s="3"/>
       <c r="H51" s="20"/>
     </row>
-    <row r="52" spans="2:8" ht="27" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="52" spans="2:8" ht="27" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
+  <autoFilter ref="B8:H23" xr:uid="{00000000-0001-0000-0200-000000000000}">
+    <filterColumn colId="6">
+      <filters>
+        <filter val="Campestre"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B9:I23">
     <sortCondition ref="B9:B23"/>
   </sortState>

</xml_diff>